<commit_message>
auto: snapshot 2026-07-25 05:30:27
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -463,11 +463,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-25 13:00:10</t>
+          <t>Timestamp: 2026-07-25 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>33366</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="3">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1560</v>
+        <v>1680</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>1240</v>
+        <v>1306</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>931</v>
+        <v>1051</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>2875</v>
+        <v>2995</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>2200</v>
+        <v>2500</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>3864</v>
+        <v>3984</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>1550</v>
+        <v>2110</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>2670</v>
+        <v>2790</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>2584</v>
+        <v>2704</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>1020</v>
+        <v>1140</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:00:00
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="2026-07-25" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1259,4 +1260,832 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-26 13:00:00</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>73429</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>228</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>9021</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>253</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>12288</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+2880</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5463</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>12665</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+3600</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>4503</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+2823</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+444</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5816</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1101</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3991</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+2940</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5615</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2620</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>7404</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1920</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>6520</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+4020</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>8101</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4480</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8127</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+4143</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>3795</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1685</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>4786</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2680</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>5460</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>4266</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+241</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>3851</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+1061</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>5065</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+2640</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>2252</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10316</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+3184</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>5347</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+1063</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>2573</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>4540</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+4540</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1470</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 210$</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>645</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>3438</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+1143</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>4084</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1380</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>14355</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+3284</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>6894</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>3514</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>5881</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+4741</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21569</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+5645</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>749</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+404</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>791</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2561</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+1261</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:30:12
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -1292,11 +1292,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:00:12</t>
+          <t>Timestamp: 2026-07-26 13:30:12</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>73429</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="3">
@@ -1563,11 +1563,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>3991</v>
+        <v>4291</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+2940</t>
+          <t>+3240</t>
         </is>
       </c>
     </row>
@@ -1578,11 +1578,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>5615</v>
+        <v>6215</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+2620</t>
+          <t>+3220</t>
         </is>
       </c>
     </row>
@@ -1638,11 +1638,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>6520</v>
+        <v>6760</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+4020</t>
+          <t>+4260</t>
         </is>
       </c>
     </row>
@@ -1668,11 +1668,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>8101</v>
+        <v>8461</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+2160</t>
         </is>
       </c>
     </row>
@@ -1833,11 +1833,11 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>10316</v>
+        <v>10336</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>+3184</t>
+          <t>+3204</t>
         </is>
       </c>
     </row>
@@ -1953,11 +1953,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>14355</v>
+        <v>14715</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+3284</t>
+          <t>+3644</t>
         </is>
       </c>
     </row>
@@ -2013,11 +2013,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>21569</v>
+        <v>21929</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+5645</t>
+          <t>+6005</t>
         </is>
       </c>
     </row>
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>749</v>
+        <v>989</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+404</t>
+          <t>+644</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="2026-07-25" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2088,4 +2089,832 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-27 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>54978</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>228</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>9895</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+874</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>253</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>13128</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5463</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>14045</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1380</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>4503</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2740</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5816</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>8122</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3831</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>6215</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>8004</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>9900</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+3140</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>9521</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4480</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1670</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>12679</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+4552</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>3795</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4786</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5460</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>4266</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>6621</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+2770</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>9751</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+4686</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2252</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>15154</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+4818</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>5347</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>3073</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1470</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 210$</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+2862</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>4028</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+590</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>6834</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+2750</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>19639</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+4924</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>7694</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>3914</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>8891</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+3010</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>25109</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+3180</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+481</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>3071</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:30:21
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -2097,7 +2097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2121,11 +2121,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-27 13:00:09</t>
+          <t>Timestamp: 2026-07-27 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54978</v>
+        <v>543</v>
       </c>
     </row>
     <row r="3">
@@ -2197,11 +2197,11 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>13128</v>
+        <v>13188</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -2392,11 +2392,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>8122</v>
+        <v>8182</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3831</t>
+          <t>+3891</t>
         </is>
       </c>
     </row>
@@ -2437,11 +2437,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>8004</v>
+        <v>8064</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+660</t>
         </is>
       </c>
     </row>
@@ -2542,11 +2542,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>12679</v>
+        <v>12739</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+4552</t>
+          <t>+4612</t>
         </is>
       </c>
     </row>
@@ -2632,11 +2632,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>6621</v>
+        <v>6681</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+2770</t>
+          <t>+2830</t>
         </is>
       </c>
     </row>
@@ -2647,11 +2647,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>9751</v>
+        <v>9811</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+4686</t>
+          <t>+4746</t>
         </is>
       </c>
     </row>
@@ -2677,11 +2677,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>15154</v>
+        <v>15157</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+4818</t>
+          <t>+4821</t>
         </is>
       </c>
     </row>
@@ -2767,11 +2767,11 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>6834</v>
+        <v>6894</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>+2750</t>
+          <t>+2810</t>
         </is>
       </c>
     </row>
@@ -2782,11 +2782,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>19639</v>
+        <v>19699</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+4924</t>
+          <t>+4984</t>
         </is>
       </c>
     </row>
@@ -2823,88 +2823,103 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Anbu Zannpist</t>
+          <t>SS HaN</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>8891</v>
+        <v>0</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+3010</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>xZenny V</t>
+          <t>Anbu Zannpist</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>25109</v>
+        <v>8891</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+3180</t>
+          <t>+3010</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>SS Rain</t>
+          <t>xZenny V</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>1469</v>
+        <v>25109</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+3180</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Ruzzz</t>
+          <t>SS Rain</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>1272</v>
+        <v>1469</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+481</t>
+          <t>+480</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>geri</t>
+          <t>Ruzzz</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>3071</v>
+        <v>1272</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>+510</t>
+          <t>+481</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>3131</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+570</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
           <t>SS Aiko</t>
         </is>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B55" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026-07-25" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2932,4 +2933,862 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-28 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>23778</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>303</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>10335</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+440</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>328</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>14760</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+1572</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5698</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+235</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>15028</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+983</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+110</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>4503</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>3340</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5996</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+180</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>10092</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1910</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>6215</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>8556</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+492</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>11346</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1446</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>10071</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4650</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>2120</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>14315</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1576</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>4095</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4786</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5670</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>4476</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>7541</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11468</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1657</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2262</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>16073</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+916</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>5517</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>3198</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>315</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1470</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 210$</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>4217</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>4088</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+60</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>6969</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>21563</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+1864</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8172</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+478</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4214</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>801</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+801</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>10256</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+1365</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>26604</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+1495</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1522</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>3131</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -2965,11 +2965,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:00:09</t>
+          <t>Timestamp: 2026-07-28 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>23778</v>
+        <v>535</v>
       </c>
     </row>
     <row r="3">
@@ -3071,11 +3071,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>15028</v>
+        <v>15058</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+983</t>
+          <t>+1013</t>
         </is>
       </c>
     </row>
@@ -3206,11 +3206,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5996</v>
+        <v>6046</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+180</t>
+          <t>+230</t>
         </is>
       </c>
     </row>
@@ -3236,11 +3236,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>10092</v>
+        <v>10122</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+1910</t>
+          <t>+1940</t>
         </is>
       </c>
     </row>
@@ -3356,11 +3356,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>4650</v>
+        <v>4700</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+170</t>
+          <t>+220</t>
         </is>
       </c>
     </row>
@@ -3386,11 +3386,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>14315</v>
+        <v>14345</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1576</t>
+          <t>+1606</t>
         </is>
       </c>
     </row>
@@ -3431,11 +3431,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>5670</v>
+        <v>5720</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+210</t>
+          <t>+260</t>
         </is>
       </c>
     </row>
@@ -3446,11 +3446,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>4476</v>
+        <v>4526</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+210</t>
+          <t>+260</t>
         </is>
       </c>
     </row>
@@ -3476,11 +3476,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>7541</v>
+        <v>7571</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+890</t>
         </is>
       </c>
     </row>
@@ -3491,11 +3491,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>11468</v>
+        <v>11498</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+1657</t>
+          <t>+1687</t>
         </is>
       </c>
     </row>
@@ -3521,11 +3521,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>16073</v>
+        <v>16103</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+916</t>
+          <t>+946</t>
         </is>
       </c>
     </row>
@@ -3536,11 +3536,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>5517</v>
+        <v>5567</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+170</t>
+          <t>+220</t>
         </is>
       </c>
     </row>
@@ -3641,11 +3641,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>21563</v>
+        <v>21593</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1864</t>
+          <t>+1894</t>
         </is>
       </c>
     </row>
@@ -3686,11 +3686,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>801</v>
+        <v>876</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+801</t>
+          <t>+876</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:00:12
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -11,6 +11,7 @@
     <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3791,4 +3792,862 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-29 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>378</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>11306</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+971</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>478</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>14910</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6408</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>15088</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1370</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>4653</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>3995</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+655</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>6559</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+513</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>11742</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1620</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>6365</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>8706</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>12227</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+881</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>10495</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5200</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>2626</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+506</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>15435</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1090</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>4095</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4786</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6420</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>5126</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>8391</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>12502</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1004</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2272</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>17076</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+973</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>6097</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+530</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>3318</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+120</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>975</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1746</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+276</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>5083</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>4088</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>7394</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>23199</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+1606</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8818</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+646</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4369</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+155</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>1371</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+495</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>10706</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>27289</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+685</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1602</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+80</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>3231</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:30:24
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -3824,11 +3824,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:00:11</t>
+          <t>Timestamp: 2026-07-29 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>523</v>
       </c>
     </row>
     <row r="3">
@@ -3915,11 +3915,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>6408</v>
+        <v>6438</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+740</t>
         </is>
       </c>
     </row>
@@ -4050,11 +4050,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>3995</v>
+        <v>4103</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+655</t>
+          <t>+763</t>
         </is>
       </c>
     </row>
@@ -4065,11 +4065,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>6559</v>
+        <v>6594</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+513</t>
+          <t>+548</t>
         </is>
       </c>
     </row>
@@ -4095,11 +4095,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>11742</v>
+        <v>11802</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+1620</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -4125,11 +4125,11 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+50</t>
         </is>
       </c>
     </row>
@@ -4215,11 +4215,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>5200</v>
+        <v>5230</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+530</t>
         </is>
       </c>
     </row>
@@ -4245,11 +4245,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>15435</v>
+        <v>15465</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1090</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -4290,11 +4290,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>6420</v>
+        <v>6450</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+730</t>
         </is>
       </c>
     </row>
@@ -4350,11 +4350,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>12502</v>
+        <v>12532</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+1004</t>
+          <t>+1034</t>
         </is>
       </c>
     </row>
@@ -4380,11 +4380,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>17076</v>
+        <v>17106</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+973</t>
+          <t>+1003</t>
         </is>
       </c>
     </row>
@@ -4395,11 +4395,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>6097</v>
+        <v>6127</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+530</t>
+          <t>+560</t>
         </is>
       </c>
     </row>
@@ -4500,11 +4500,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>23199</v>
+        <v>23229</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1606</t>
+          <t>+1636</t>
         </is>
       </c>
     </row>
@@ -4515,11 +4515,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>8818</v>
+        <v>8848</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+646</t>
+          <t>+676</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4650,4 +4651,877 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-30 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>19373</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>528</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>11456</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>628</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>14910</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7098</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>15088</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1520</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>4803</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5140</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1037</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>7181</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+587</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>13403</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1601</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9151</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+445</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>13127</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>10795</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>5846</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+616</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>3286</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>16541</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1076</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4250</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+155</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>4886</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7102</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+652</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>5530</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+404</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>8591</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>13663</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+1131</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2277</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18320</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>6735</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+608</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3443</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+306</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1896</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>5499</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+416</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4238</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>7544</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>24835</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1606</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>9907</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1059</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>4509</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+140</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>1601</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+230</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>11257</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+551</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>27769</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1602</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>3336</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+105</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:30:22
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -4683,11 +4683,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:00:11</t>
+          <t>Timestamp: 2026-07-30 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19373</v>
+        <v>19808</v>
       </c>
     </row>
     <row r="3">
@@ -4774,11 +4774,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>7098</v>
+        <v>7130</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+692</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -4924,11 +4924,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5140</v>
+        <v>5149</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+1037</t>
+          <t>+1046</t>
         </is>
       </c>
     </row>
@@ -4939,11 +4939,11 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>7181</v>
+        <v>7211</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+617</t>
         </is>
       </c>
     </row>
@@ -4969,11 +4969,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>13403</v>
+        <v>13433</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+1601</t>
+          <t>+1631</t>
         </is>
       </c>
     </row>
@@ -5089,11 +5089,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>5846</v>
+        <v>5876</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+616</t>
+          <t>+646</t>
         </is>
       </c>
     </row>
@@ -5104,11 +5104,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>3286</v>
+        <v>3361</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+735</t>
         </is>
       </c>
     </row>
@@ -5164,11 +5164,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>7102</v>
+        <v>7132</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+652</t>
+          <t>+682</t>
         </is>
       </c>
     </row>
@@ -5179,11 +5179,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>5530</v>
+        <v>5560</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+404</t>
+          <t>+434</t>
         </is>
       </c>
     </row>
@@ -5254,11 +5254,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>18320</v>
+        <v>18350</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1214</t>
+          <t>+1244</t>
         </is>
       </c>
     </row>
@@ -5269,11 +5269,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>6735</v>
+        <v>6765</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+608</t>
+          <t>+638</t>
         </is>
       </c>
     </row>
@@ -5374,11 +5374,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>24835</v>
+        <v>24865</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+1606</t>
+          <t>+1636</t>
         </is>
       </c>
     </row>
@@ -5389,11 +5389,11 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>9907</v>
+        <v>9937</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+1059</t>
+          <t>+1089</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:46:41
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -4683,11 +4683,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:30:22</t>
+          <t>Timestamp: 2026-07-30 13:46:41</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19808</v>
+        <v>19965</v>
       </c>
     </row>
     <row r="3">
@@ -4774,11 +4774,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>7130</v>
+        <v>7134</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+692</t>
+          <t>+696</t>
         </is>
       </c>
     </row>
@@ -4924,11 +4924,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5149</v>
+        <v>5152</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+1046</t>
+          <t>+1049</t>
         </is>
       </c>
     </row>
@@ -4939,11 +4939,11 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>7211</v>
+        <v>7241</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>+617</t>
+          <t>+647</t>
         </is>
       </c>
     </row>
@@ -5089,11 +5089,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>5876</v>
+        <v>5906</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+646</t>
+          <t>+676</t>
         </is>
       </c>
     </row>
@@ -5164,11 +5164,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>7132</v>
+        <v>7162</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+682</t>
+          <t>+712</t>
         </is>
       </c>
     </row>
@@ -5179,11 +5179,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>5560</v>
+        <v>5590</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+434</t>
+          <t>+464</t>
         </is>
       </c>
     </row>
@@ -5269,11 +5269,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>6765</v>
+        <v>6795</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+638</t>
+          <t>+668</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -13,6 +13,7 @@
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5524,4 +5525,877 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-31 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>603</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>11590</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+134</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>703</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>15930</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7342</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+208</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>15088</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1670</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+335</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5684</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+532</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>7533</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+292</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>14439</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1006</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9842</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+691</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>14156</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1029</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>10945</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6124</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+218</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>3796</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+435</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>17664</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1123</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4250</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+190</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7316</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+154</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>5726</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+136</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>8691</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>14546</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+883</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2277</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>19254</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+904</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7063</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+268</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3443</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1748</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+467</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2030</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+134</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>5949</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4238</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>7620</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+76</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>26251</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1386</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>10617</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>4609</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>1826</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>11842</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+585</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>28435</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+666</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1652</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>3502</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+166</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:30:30
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -5557,11 +5557,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-31 13:00:10</t>
+          <t>Timestamp: 2026-07-31 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3">
@@ -5798,11 +5798,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5684</v>
+        <v>5712</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+532</t>
+          <t>+560</t>
         </is>
       </c>
     </row>
@@ -5918,11 +5918,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>14156</v>
+        <v>14216</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+1029</t>
+          <t>+1089</t>
         </is>
       </c>
     </row>
@@ -6248,11 +6248,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>26251</v>
+        <v>26311</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+1386</t>
+          <t>+1446</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:00:14
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6398,4 +6399,877 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-01 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>21103</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>753</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>11590</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>853</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>16890</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+440</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>15088</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1970</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>930</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>6458</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+746</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+593</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1310</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>15310</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+871</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9842</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Oksihina</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>15476</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1260</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>11079</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+134</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6726</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+602</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>5264</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1468</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>18450</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+786</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4260</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7696</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>8891</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>14547</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2277</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>19424</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+431</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3693</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2072</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+324</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2030</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>7239</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4238</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>7770</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>28246</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1935</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>10617</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>4609</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+201</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>12394</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+552</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>34026</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+5591</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1652</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>3502</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:30:29
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -6431,11 +6431,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-01 13:00:13</t>
+          <t>Timestamp: 2026-08-01 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>21103</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3">
@@ -6867,11 +6867,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>18450</v>
+        <v>18453</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+786</t>
+          <t>+789</t>
         </is>
       </c>
     </row>
@@ -7167,11 +7167,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>2027</v>
+        <v>2267</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+201</t>
+          <t>+441</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:30:24
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -7305,11 +7305,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-02 13:00:11</t>
+          <t>Timestamp: 2026-08-02 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>21934</v>
+        <v>698</v>
       </c>
     </row>
     <row r="3">
@@ -7456,11 +7456,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1974</v>
+        <v>2035</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1584</t>
+          <t>+1645</t>
         </is>
       </c>
     </row>
@@ -7471,11 +7471,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>930</v>
+        <v>1080</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -7546,11 +7546,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>6890</v>
+        <v>6898</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+432</t>
+          <t>+440</t>
         </is>
       </c>
     </row>
@@ -7666,11 +7666,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>16796</v>
+        <v>16946</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1470</t>
         </is>
       </c>
     </row>
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>4238</v>
+        <v>4508</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+270</t>
         </is>
       </c>
     </row>
@@ -7996,11 +7996,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>30772</v>
+        <v>30832</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+2526</t>
+          <t>+2586</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:00:12
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16,6 +16,7 @@
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1269,6 +1270,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-03 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>64785</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+141</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12110</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+220</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1153</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>18881</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+1401</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>18166</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2538</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>311</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+141</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2570</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>3370</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1335</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1140</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+60</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>7262</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+364</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>16855</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1035</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>10143</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+301</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>165</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+165</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>18392</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1446</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>13097</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6726</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>8095</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1881</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>21437</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4680</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7696</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>17753</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+8662</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>15138</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2507</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+130</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>22249</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+521</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3943</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>4422</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+1972</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2294</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+264</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>10279</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1599</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4698</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+190</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8680</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>33583</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2751</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>12689</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>4939</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>3913</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+831</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>13956</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+1092</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>35808</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+582</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>2397</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3752</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>28548</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:30:24
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -1300,11 +1300,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:00:11</t>
+          <t>Timestamp: 2026-08-03 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>64785</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3">
@@ -1451,11 +1451,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>3370</v>
+        <v>3400</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1335</t>
+          <t>+1365</t>
         </is>
       </c>
     </row>
@@ -1541,11 +1541,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>7262</v>
+        <v>7279</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+364</t>
+          <t>+381</t>
         </is>
       </c>
     </row>
@@ -1991,11 +1991,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>33583</v>
+        <v>33635</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+2751</t>
+          <t>+2803</t>
         </is>
       </c>
     </row>
@@ -2111,11 +2111,11 @@
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>2397</v>
+        <v>2447</v>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+410</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -17,6 +17,7 @@
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2158,6 +2159,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-04 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12151</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12410</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1153</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>19401</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+520</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>19124</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+958</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>311</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2720</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4596</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1196</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1215</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>7744</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+465</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>17255</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>10443</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>165</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>19292</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+110</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>13565</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+468</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6726</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>8320</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>21678</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+241</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4685</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7696</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>17973</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+220</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>15313</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+175</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2507</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>22586</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+337</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>4154</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+211</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>5172</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2294</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>10729</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4773</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8732</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+52</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>35033</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1398</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>12689</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>5039</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>4543</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>14421</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+465</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>36259</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+451</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>2597</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3852</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>28548</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:30:26
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -2189,11 +2189,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:00:10</t>
+          <t>Timestamp: 2026-08-04 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>12151</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -2340,11 +2340,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>4596</v>
+        <v>4626</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1196</t>
+          <t>+1226</t>
         </is>
       </c>
     </row>
@@ -2430,11 +2430,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>7744</v>
+        <v>7758</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+465</t>
+          <t>+479</t>
         </is>
       </c>
     </row>
@@ -2880,11 +2880,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>35033</v>
+        <v>35063</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+1398</t>
+          <t>+1428</t>
         </is>
       </c>
     </row>
@@ -2970,11 +2970,11 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>36259</v>
+        <v>36349</v>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>+451</t>
+          <t>+541</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:00:12
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -18,6 +18,7 @@
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3047,6 +3048,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-05 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>11641</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12410</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1153</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>20121</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>20122</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+998</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>311</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2870</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>5970</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1344</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1215</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>8165</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+407</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>17750</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+495</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6540</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>10593</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>20207</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+915</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>14007</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+442</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6726</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>8931</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+611</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>22068</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+390</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4685</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7696</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>18069</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+96</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>15493</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+180</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2517</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>22928</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+342</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>4404</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>5995</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+823</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2294</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>11044</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+315</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4773</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8817</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>36065</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>12849</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+160</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>5139</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>4831</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+288</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>14961</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>36739</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+390</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>2796</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3852</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>28548</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:30:29
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -3078,11 +3078,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-05 13:00:12</t>
+          <t>Timestamp: 2026-08-05 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>11641</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3">
@@ -3229,11 +3229,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>5970</v>
+        <v>6000</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1344</t>
+          <t>+1374</t>
         </is>
       </c>
     </row>
@@ -3319,11 +3319,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>8165</v>
+        <v>8195</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+437</t>
         </is>
       </c>
     </row>
@@ -3784,11 +3784,11 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>12849</v>
+        <v>12879</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+160</t>
+          <t>+190</t>
         </is>
       </c>
     </row>
@@ -3889,11 +3889,11 @@
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>2796</v>
+        <v>2947</v>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>+199</t>
+          <t>+350</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -19,6 +19,7 @@
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3936,6 +3937,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-06 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12814</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1110</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12542</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+132</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1228</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>21069</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+948</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>21127</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1005</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>386</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS|Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>3002</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>7356</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1356</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>8608</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+413</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>18725</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+975</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>6540</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>11035</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+442</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>21092</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+885</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>14153</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+146</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6726</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>9607</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+676</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>22338</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+270</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4835</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7696</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>18247</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+178</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>15663</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2517</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>23118</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+190</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>4529</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>6594</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2579</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+285</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>11044</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4773</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8922</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+105</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>37405</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1340</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>13155</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+276</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>5139</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5191</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>15329</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+368</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>36739</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>3749</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+802</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3852</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>28548</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:00:08
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -20,6 +20,7 @@
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4825,6 +4826,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-07 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>17730</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12844</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+302</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1378</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>22374</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+1305</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>23083</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1956</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>386</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS|Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>3302</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>9126</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1740</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>kralBarKaha</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5138</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>885</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>9278</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+656</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>19457</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+732</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>6540</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>11335</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>22457</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1365</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>RS | ÐICTATØR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1125</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D e a D L S o u L</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>14453</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>6726</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>10753</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1146</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>23238</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4985</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>B a r K a H a</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5076</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7696</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>18247</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>15813</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2517</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>23493</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>4654</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>6744</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2579</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>11571</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+527</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>4773</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8997</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>39555</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2120</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>13649</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+494</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>5339</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5533</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+295</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>15629</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>36739</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>3949</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3852</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>28548</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:18:48
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -4856,11 +4856,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:00:08</t>
+          <t>Timestamp: 2026-08-07 13:18:48</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>17730</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -5007,11 +5007,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>9126</v>
+        <v>9156</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1740</t>
+          <t>+1770</t>
         </is>
       </c>
     </row>
@@ -5037,11 +5037,11 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>5138</v>
+        <v>5168</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+30</t>
         </is>
       </c>
     </row>
@@ -5082,11 +5082,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>9278</v>
+        <v>9292</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+656</t>
+          <t>+670</t>
         </is>
       </c>
     </row>
@@ -5202,11 +5202,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>22457</v>
+        <v>22487</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+1365</t>
+          <t>+1395</t>
         </is>
       </c>
     </row>
@@ -5292,11 +5292,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>23238</v>
+        <v>23268</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+930</t>
         </is>
       </c>
     </row>
@@ -5547,11 +5547,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>39555</v>
+        <v>39585</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+2120</t>
+          <t>+2150</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:30:29
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -4856,11 +4856,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:18:48</t>
+          <t>Timestamp: 2026-08-07 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3">
@@ -5082,11 +5082,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>9292</v>
+        <v>9295</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+673</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:49:00
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -4856,11 +4856,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:30:28</t>
+          <t>Timestamp: 2026-08-07 13:48:59</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>167</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3">
@@ -5007,11 +5007,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>9156</v>
+        <v>9186</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1770</t>
+          <t>+1800</t>
         </is>
       </c>
     </row>
@@ -5082,11 +5082,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>9295</v>
+        <v>9298</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+673</t>
+          <t>+676</t>
         </is>
       </c>
     </row>
@@ -5202,11 +5202,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>22487</v>
+        <v>22517</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+1395</t>
+          <t>+1425</t>
         </is>
       </c>
     </row>
@@ -5547,11 +5547,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>39585</v>
+        <v>39615</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+2150</t>
+          <t>+2180</t>
         </is>
       </c>
     </row>
@@ -5592,11 +5592,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>5533</v>
+        <v>5608</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+295</t>
+          <t>+370</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:02:02
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -5745,11 +5745,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:00:11</t>
+          <t>Timestamp: 2026-08-08 13:02:02</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>22089</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:30:22
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -5745,11 +5745,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:02:02</t>
+          <t>Timestamp: 2026-08-08 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3">
@@ -5896,11 +5896,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>11572</v>
+        <v>11692</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+2386</t>
+          <t>+2506</t>
         </is>
       </c>
     </row>
@@ -5911,11 +5911,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>5478</v>
+        <v>5698</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+310</t>
+          <t>+530</t>
         </is>
       </c>
     </row>
@@ -6091,11 +6091,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>1971</v>
+        <v>2271</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+846</t>
+          <t>+1146</t>
         </is>
       </c>
     </row>
@@ -6166,11 +6166,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>24039</v>
+        <v>24279</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+771</t>
+          <t>+1011</t>
         </is>
       </c>
     </row>
@@ -6421,11 +6421,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>42165</v>
+        <v>42285</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2670</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:32:18
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -5745,11 +5745,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:30:22</t>
+          <t>Timestamp: 2026-08-08 13:32:18</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1000</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="3">
@@ -6271,11 +6271,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>15813</v>
+        <v>16273</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+460</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-09 05:00:06
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -22,6 +22,7 @@
     <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6603,6 +6604,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-09 13:00:05</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>728375</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>16400</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+15140</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4161</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>20162</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+6958</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+14624</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>43858</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+20224</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>12935</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+5153</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>38330</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+13243</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>13488</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+13102</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>15853</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+12251</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Cut Nyak Dhien</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>29759</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+18067</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Akame</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5248</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>19190</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+18305</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>22349</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+13001</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>14108</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+12478</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>44453</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+22833</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>25165</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+18334</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>10557</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+10389</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>28961</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+16666</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>19113</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+18898</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ðreey</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>44771</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+20706</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>×SAMANEA×</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>6298</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>RS | ÐICTATØR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>22111</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+19840</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>14727</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>9879</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+3153</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>16398</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+4319</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>40598</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+16319</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>14169</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+8864</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>11147</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+3451</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>For Sale</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6928</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+822</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7669</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+5399</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>68179</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+49732</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>29489</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+13216</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>17255</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+14678</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>31120</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+7182</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>10122</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+2628</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>23334</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+18680</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>24442</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+17658</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>9147</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+6568</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>32034</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+20163</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>17206</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+12133</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>16865</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+7658</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>63622</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+21337</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>34579</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+20730</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>18310</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+12771</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>13779</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+7681</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Zannpist</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>32578</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+16029</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>54928</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+18189</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kee Cap M</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>13014</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>10032</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+8563</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>21521</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+17222</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>13580</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+9728</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>11677</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+11677</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>77040</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+48492</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-09 05:13:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -6634,11 +6634,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-09 13:00:05</t>
+          <t>Timestamp: 2026-08-09 13:13:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>728375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -23,6 +23,7 @@
     <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7492,6 +7493,864 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-10 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>9795</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>372</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>362</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka New</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>462</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>322</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>632</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>411</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>JBT.Kage</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>687</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>INA|Réxx</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>873</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>934</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Kappa</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>866</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>186</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>499</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:30:31
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -7523,11 +7523,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-10 13:00:08</t>
+          <t>Timestamp: 2026-08-10 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9795</v>
+        <v>714</v>
       </c>
     </row>
     <row r="3">
@@ -7614,7 +7614,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>372</v>
+        <v>396</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -7689,7 +7689,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>462</v>
+        <v>612</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -7764,7 +7764,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>322</v>
+        <v>472</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
@@ -7809,7 +7809,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>632</v>
+        <v>782</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -8019,7 +8019,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>866</v>
+        <v>938</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -8244,7 +8244,7 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>100</v>
+        <v>280</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:56:08
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -7523,11 +7523,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-10 13:30:30</t>
+          <t>Timestamp: 2026-08-10 13:56:07</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>714</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="3">
@@ -7689,7 +7689,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>612</v>
+        <v>720</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -7764,7 +7764,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>472</v>
+        <v>580</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
@@ -7809,7 +7809,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>782</v>
+        <v>805</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -8184,7 +8184,7 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>1080</v>
+        <v>1152</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -24,6 +24,7 @@
     <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8351,6 +8352,879 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-11 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>31046</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1796</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1641</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1010</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>872</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2508</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+168</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3890</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3310</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>3767</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+2962</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>2837</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2426</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>3771</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS~Genny~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>2013</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1973</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+1039</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+115</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>315</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1924</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+986</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Kaidenz</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1322</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+1136</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+536</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3297</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+3297</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>660</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>2963</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+1811</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>784</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+504</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:30:19
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -8382,11 +8382,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-11 13:00:09</t>
+          <t>Timestamp: 2026-08-11 13:30:19</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>31046</v>
+        <v>740</v>
       </c>
     </row>
     <row r="3">
@@ -8548,7 +8548,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2508</v>
+        <v>2578</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -8653,11 +8653,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>3890</v>
+        <v>3960</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3310</t>
+          <t>+3380</t>
         </is>
       </c>
     </row>
@@ -8728,11 +8728,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>2837</v>
+        <v>2907</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2426</t>
+          <t>+2496</t>
         </is>
       </c>
     </row>
@@ -8743,7 +8743,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>3771</v>
+        <v>3841</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
@@ -8998,11 +8998,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>3297</v>
+        <v>3367</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+3297</t>
+          <t>+3367</t>
         </is>
       </c>
     </row>
@@ -9043,11 +9043,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>2963</v>
+        <v>3103</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+1811</t>
+          <t>+1951</t>
         </is>
       </c>
     </row>
@@ -9163,7 +9163,7 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:36:48
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -8382,11 +8382,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-11 13:30:19</t>
+          <t>Timestamp: 2026-08-11 13:36:48</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>740</v>
+        <v>801</v>
       </c>
     </row>
     <row r="3">
@@ -8548,7 +8548,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2578</v>
+        <v>2639</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -9256,11 +9256,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:00:11</t>
+          <t>Timestamp: 2026-08-12 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>32397</v>
+        <v>747</v>
       </c>
     </row>
     <row r="3">
@@ -9347,11 +9347,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>3626</v>
+        <v>3926</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+1830</t>
+          <t>+2130</t>
         </is>
       </c>
     </row>
@@ -9497,11 +9497,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>762</v>
+        <v>789</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+762</t>
+          <t>+789</t>
         </is>
       </c>
     </row>
@@ -9542,11 +9542,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>7214</v>
+        <v>7284</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+3254</t>
+          <t>+3324</t>
         </is>
       </c>
     </row>
@@ -9677,11 +9677,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>3553</v>
+        <v>3623</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1580</t>
+          <t>+1650</t>
         </is>
       </c>
     </row>
@@ -9767,11 +9767,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>3490</v>
+        <v>3560</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1566</t>
+          <t>+1636</t>
         </is>
       </c>
     </row>
@@ -9872,11 +9872,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>6540</v>
+        <v>6610</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+3173</t>
+          <t>+3243</t>
         </is>
       </c>
     </row>
@@ -9887,11 +9887,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>2012</v>
+        <v>2082</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+1352</t>
+          <t>+1422</t>
         </is>
       </c>
     </row>
@@ -9917,11 +9917,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>5044</v>
+        <v>5114</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+1941</t>
+          <t>+2011</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:58:03
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -9256,11 +9256,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:30:22</t>
+          <t>Timestamp: 2026-08-12 13:58:02</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>747</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="3">
@@ -9422,11 +9422,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>4774</v>
+        <v>4974</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+2135</t>
+          <t>+2335</t>
         </is>
       </c>
     </row>
@@ -9497,11 +9497,11 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>+789</t>
+          <t>+794</t>
         </is>
       </c>
     </row>
@@ -9542,11 +9542,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>7284</v>
+        <v>7354</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+3324</t>
+          <t>+3394</t>
         </is>
       </c>
     </row>
@@ -9617,11 +9617,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>5247</v>
+        <v>5387</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2340</t>
+          <t>+2480</t>
         </is>
       </c>
     </row>
@@ -9677,11 +9677,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>3623</v>
+        <v>3693</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1650</t>
+          <t>+1720</t>
         </is>
       </c>
     </row>
@@ -9767,11 +9767,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>3560</v>
+        <v>3630</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1636</t>
+          <t>+1706</t>
         </is>
       </c>
     </row>
@@ -9872,11 +9872,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>6610</v>
+        <v>6680</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+3243</t>
+          <t>+3313</t>
         </is>
       </c>
     </row>
@@ -9887,11 +9887,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>2082</v>
+        <v>2152</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+1422</t>
+          <t>+1492</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -26,6 +26,7 @@
     <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10927,6 +10928,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-13 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>32122</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5016</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1090</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>4691</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1142</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1180</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1172</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>7428</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+2454</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1959</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+1165</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>915</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+535</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>10502</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3148</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>510</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>7593</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+2420</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>7657</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2270</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>8688</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2477</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5573</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1880</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>510</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>435</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>685</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>5840</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2210</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>3236</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1771</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>9846</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3166</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2682</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+530</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>6445</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+1331</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>1596</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>2731</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+1271</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:18:35
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -10958,11 +10958,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:00:10</t>
+          <t>Timestamp: 2026-08-13 13:18:34</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>32122</v>
+        <v>487</v>
       </c>
     </row>
     <row r="3">
@@ -11124,11 +11124,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>7428</v>
+        <v>7498</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+2454</t>
+          <t>+2524</t>
         </is>
       </c>
     </row>
@@ -11184,11 +11184,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>1959</v>
+        <v>1975</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+1165</t>
+          <t>+1181</t>
         </is>
       </c>
     </row>
@@ -11229,11 +11229,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>10502</v>
+        <v>10554</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3148</t>
+          <t>+3200</t>
         </is>
       </c>
     </row>
@@ -11274,11 +11274,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>7593</v>
+        <v>7663</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+2420</t>
+          <t>+2490</t>
         </is>
       </c>
     </row>
@@ -11319,11 +11319,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>8688</v>
+        <v>8758</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2477</t>
+          <t>+2547</t>
         </is>
       </c>
     </row>
@@ -11349,11 +11349,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>5573</v>
+        <v>5643</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+1880</t>
+          <t>+1950</t>
         </is>
       </c>
     </row>
@@ -11529,11 +11529,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>3236</v>
+        <v>3306</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1771</t>
+          <t>+1841</t>
         </is>
       </c>
     </row>
@@ -11544,11 +11544,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>9846</v>
+        <v>9916</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3166</t>
+          <t>+3236</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -10958,11 +10958,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:18:34</t>
+          <t>Timestamp: 2026-08-13 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>487</v>
+        <v>558</v>
       </c>
     </row>
     <row r="3">
@@ -11184,11 +11184,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>1975</v>
+        <v>1976</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+1181</t>
+          <t>+1182</t>
         </is>
       </c>
     </row>
@@ -11439,11 +11439,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>5840</v>
+        <v>5910</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2210</t>
+          <t>+2280</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:48:47
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -10958,11 +10958,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:30:23</t>
+          <t>Timestamp: 2026-08-13 13:48:46</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>558</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="3">
@@ -11124,11 +11124,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>7498</v>
+        <v>7568</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+2524</t>
+          <t>+2594</t>
         </is>
       </c>
     </row>
@@ -11184,11 +11184,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>1976</v>
+        <v>1991</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+1182</t>
+          <t>+1197</t>
         </is>
       </c>
     </row>
@@ -11229,11 +11229,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>10554</v>
+        <v>10624</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3200</t>
+          <t>+3270</t>
         </is>
       </c>
     </row>
@@ -11274,11 +11274,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>7663</v>
+        <v>7733</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+2490</t>
+          <t>+2560</t>
         </is>
       </c>
     </row>
@@ -11349,11 +11349,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>5643</v>
+        <v>5713</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+1950</t>
+          <t>+2020</t>
         </is>
       </c>
     </row>
@@ -11439,11 +11439,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>5910</v>
+        <v>5980</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2280</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -11469,11 +11469,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>1993</v>
+        <v>2275</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+282</t>
         </is>
       </c>
     </row>
@@ -11529,11 +11529,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>3306</v>
+        <v>3376</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1841</t>
+          <t>+1911</t>
         </is>
       </c>
     </row>
@@ -11544,11 +11544,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>9916</v>
+        <v>9986</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3236</t>
+          <t>+3306</t>
         </is>
       </c>
     </row>
@@ -11589,11 +11589,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>6445</v>
+        <v>6645</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+1331</t>
+          <t>+1531</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -27,6 +27,7 @@
     <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11771,6 +11772,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-14 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>23695</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5316</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>5291</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1471</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+291</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1472</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>9976</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+2408</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2872</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+881</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1085</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>13260</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+2636</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>510</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Nami</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>9887</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>9984</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2327</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>10058</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>7774</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2061</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>435</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>685</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>6680</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2595</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+320</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>3936</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>12630</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+2644</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2682</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>7643</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+998</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2086</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>3731</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -11802,11 +11802,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:00:11</t>
+          <t>Timestamp: 2026-08-14 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>23695</v>
+        <v>358</v>
       </c>
     </row>
     <row r="3">
@@ -11968,11 +11968,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>9976</v>
+        <v>10046</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+2408</t>
+          <t>+2478</t>
         </is>
       </c>
     </row>
@@ -12028,11 +12028,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>2872</v>
+        <v>2880</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+881</t>
+          <t>+889</t>
         </is>
       </c>
     </row>
@@ -12073,11 +12073,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>13260</v>
+        <v>13330</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+2636</t>
+          <t>+2706</t>
         </is>
       </c>
     </row>
@@ -12148,11 +12148,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>9984</v>
+        <v>10054</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2327</t>
+          <t>+2397</t>
         </is>
       </c>
     </row>
@@ -12193,11 +12193,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>7774</v>
+        <v>7844</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2061</t>
+          <t>+2131</t>
         </is>
       </c>
     </row>
@@ -12388,11 +12388,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>12630</v>
+        <v>12700</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2644</t>
+          <t>+2714</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:57:45
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -11802,11 +11802,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:30:23</t>
+          <t>Timestamp: 2026-08-14 13:57:44</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>358</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="3">
@@ -11848,11 +11848,11 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>222</v>
+        <v>372</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -11893,11 +11893,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>5316</v>
+        <v>5616</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -12028,11 +12028,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>2880</v>
+        <v>2886</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+889</t>
+          <t>+895</t>
         </is>
       </c>
     </row>
@@ -12073,11 +12073,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>13330</v>
+        <v>13400</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+2706</t>
+          <t>+2776</t>
         </is>
       </c>
     </row>
@@ -12118,7 +12118,7 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>9887</v>
+        <v>10187</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
@@ -12148,11 +12148,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>10054</v>
+        <v>10124</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2397</t>
+          <t>+2467</t>
         </is>
       </c>
     </row>
@@ -12163,11 +12163,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>10058</v>
+        <v>10258</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1500</t>
         </is>
       </c>
     </row>
@@ -12193,11 +12193,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>7844</v>
+        <v>7905</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2131</t>
+          <t>+2192</t>
         </is>
       </c>
     </row>
@@ -12388,11 +12388,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>12700</v>
+        <v>12770</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2714</t>
+          <t>+2784</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -28,6 +28,7 @@
     <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12615,6 +12616,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-15 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>28001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>822</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6216</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7117</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1826</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1771</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1472</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>13126</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+3080</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4419</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+1533</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2033</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+948</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>16449</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3049</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>510</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Nami</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>13102</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+2915</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>12131</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2007</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>12728</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2470</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>8975</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1070</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>435</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>685</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>7190</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2595</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>4156</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+220</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>14827</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+2057</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2682</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>8653</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+1010</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2636</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>4722</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+991</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+120</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:28:54
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -12646,11 +12646,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:00:10</t>
+          <t>Timestamp: 2026-08-15 13:28:53</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>28001</v>
+        <v>840</v>
       </c>
     </row>
     <row r="3">
@@ -12812,11 +12812,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>13126</v>
+        <v>13266</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+3080</t>
+          <t>+3220</t>
         </is>
       </c>
     </row>
@@ -12872,11 +12872,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>4419</v>
+        <v>4559</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+1533</t>
+          <t>+1673</t>
         </is>
       </c>
     </row>
@@ -12917,11 +12917,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>16449</v>
+        <v>16589</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3049</t>
+          <t>+3189</t>
         </is>
       </c>
     </row>
@@ -12962,11 +12962,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>13102</v>
+        <v>13242</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+2915</t>
+          <t>+3055</t>
         </is>
       </c>
     </row>
@@ -13007,11 +13007,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>12728</v>
+        <v>12868</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2470</t>
+          <t>+2610</t>
         </is>
       </c>
     </row>
@@ -13232,11 +13232,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>14827</v>
+        <v>14967</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2057</t>
+          <t>+2197</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:30:24
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -12646,11 +12646,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:28:53</t>
+          <t>Timestamp: 2026-08-15 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>840</v>
+        <v>844</v>
       </c>
     </row>
     <row r="3">
@@ -12872,11 +12872,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>4559</v>
+        <v>4562</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+1673</t>
+          <t>+1676</t>
         </is>
       </c>
     </row>
@@ -13232,11 +13232,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>14967</v>
+        <v>14968</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2197</t>
+          <t>+2198</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:53:56
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -12646,11 +12646,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:30:23</t>
+          <t>Timestamp: 2026-08-15 13:53:55</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>844</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="3">
@@ -12812,11 +12812,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>13266</v>
+        <v>13406</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+3220</t>
+          <t>+3360</t>
         </is>
       </c>
     </row>
@@ -12872,11 +12872,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>4562</v>
+        <v>4566</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+1676</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -12917,11 +12917,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>16589</v>
+        <v>16729</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3189</t>
+          <t>+3329</t>
         </is>
       </c>
     </row>
@@ -12962,11 +12962,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>13242</v>
+        <v>13382</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+3055</t>
+          <t>+3195</t>
         </is>
       </c>
     </row>
@@ -12992,11 +12992,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>12131</v>
+        <v>12531</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2007</t>
+          <t>+2407</t>
         </is>
       </c>
     </row>
@@ -13007,11 +13007,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>12868</v>
+        <v>13008</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2610</t>
+          <t>+2750</t>
         </is>
       </c>
     </row>
@@ -13232,11 +13232,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>14968</v>
+        <v>14974</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2198</t>
+          <t>+2204</t>
         </is>
       </c>
     </row>
@@ -13337,11 +13337,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>2636</v>
+        <v>2836</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+550</t>
+          <t>+750</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -29,6 +29,7 @@
     <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13459,6 +13460,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-16 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>88441</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>5100</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+4500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6816</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1240</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>9487</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+2370</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1771</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2584</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1112</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>20031</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+6625</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+284</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2533</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>20916</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+4187</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2910</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Nami</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>18682</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+5300</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>16996</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+4465</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>18344</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+5336</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1263</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1263</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>15843</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+6868</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1525</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>10183</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2993</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1206</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+1206</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>5995</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+3400</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>6996</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+2840</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>21313</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+6339</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>8278</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+5596</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>4583</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+4373</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>12014</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+3361</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>4376</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1540</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>560</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>6203</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+1481</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+168</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:01:43
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -13490,11 +13490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:00:10</t>
+          <t>Timestamp: 2026-08-16 13:01:42</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>88441</v>
+        <v>380</v>
       </c>
     </row>
     <row r="3">
@@ -13761,11 +13761,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>20916</v>
+        <v>21056</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+4187</t>
+          <t>+4327</t>
         </is>
       </c>
     </row>
@@ -14091,11 +14091,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>8278</v>
+        <v>8318</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+5596</t>
+          <t>+5636</t>
         </is>
       </c>
     </row>
@@ -14121,11 +14121,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>12014</v>
+        <v>12214</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+3361</t>
+          <t>+3561</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:30:24
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -13490,11 +13490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:01:42</t>
+          <t>Timestamp: 2026-08-16 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>380</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="3">
@@ -13596,11 +13596,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1240</v>
+        <v>1380</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1380</t>
         </is>
       </c>
     </row>
@@ -13656,11 +13656,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>20031</v>
+        <v>20171</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+6625</t>
+          <t>+6765</t>
         </is>
       </c>
     </row>
@@ -13806,11 +13806,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>18682</v>
+        <v>18822</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+5300</t>
+          <t>+5440</t>
         </is>
       </c>
     </row>
@@ -13836,11 +13836,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>16996</v>
+        <v>17136</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+4465</t>
+          <t>+4605</t>
         </is>
       </c>
     </row>
@@ -13851,11 +13851,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>18344</v>
+        <v>18744</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+5336</t>
+          <t>+5736</t>
         </is>
       </c>
     </row>
@@ -13866,11 +13866,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>1263</v>
+        <v>1403</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+1263</t>
+          <t>+1403</t>
         </is>
       </c>
     </row>
@@ -13911,11 +13911,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>540</v>
+        <v>740</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+740</t>
         </is>
       </c>
     </row>
@@ -13986,11 +13986,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>1206</v>
+        <v>1346</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+1206</t>
+          <t>+1346</t>
         </is>
       </c>
     </row>
@@ -14076,11 +14076,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>21313</v>
+        <v>21453</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+6339</t>
+          <t>+6479</t>
         </is>
       </c>
     </row>
@@ -14091,11 +14091,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>8318</v>
+        <v>8698</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+5636</t>
+          <t>+6016</t>
         </is>
       </c>
     </row>
@@ -14121,11 +14121,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>12214</v>
+        <v>12274</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+3561</t>
+          <t>+3621</t>
         </is>
       </c>
     </row>
@@ -14181,11 +14181,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>4376</v>
+        <v>4576</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+1540</t>
+          <t>+1740</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:31:58
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -13490,11 +13490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:30:23</t>
+          <t>Timestamp: 2026-08-16 13:31:57</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2600</v>
+        <v>2664</v>
       </c>
     </row>
     <row r="3">
@@ -13986,11 +13986,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>1346</v>
+        <v>1410</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+1346</t>
+          <t>+1410</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:55:33
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -13490,11 +13490,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:31:57</t>
+          <t>Timestamp: 2026-08-16 13:55:32</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2664</v>
+        <v>3624</v>
       </c>
     </row>
     <row r="3">
@@ -13596,11 +13596,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1380</v>
+        <v>1520</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>
@@ -13761,11 +13761,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>21056</v>
+        <v>21196</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+4327</t>
+          <t>+4467</t>
         </is>
       </c>
     </row>
@@ -13806,11 +13806,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>18822</v>
+        <v>18942</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+5440</t>
+          <t>+5560</t>
         </is>
       </c>
     </row>
@@ -13866,11 +13866,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>1403</v>
+        <v>1543</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+1403</t>
+          <t>+1543</t>
         </is>
       </c>
     </row>
@@ -13911,11 +13911,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>740</v>
+        <v>880</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+880</t>
         </is>
       </c>
     </row>
@@ -14076,11 +14076,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>21453</v>
+        <v>21593</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+6479</t>
+          <t>+6619</t>
         </is>
       </c>
     </row>
@@ -14091,11 +14091,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>8698</v>
+        <v>8838</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+6016</t>
+          <t>+6156</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -30,6 +30,7 @@
     <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14303,6 +14304,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-17 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>82903</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2462</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>5700</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>281</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+281</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7416</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2760</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>12647</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+3160</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1771</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>3746</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1162</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>26390</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+6219</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2533</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>31356</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+10160</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>4110</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Nami</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>24571</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+5629</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+60</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>21876</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+4740</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>23724</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+4980</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2984</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1441</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>21523</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+5680</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2260</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1380</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1525</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+260</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>12743</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2560</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+1380</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>9195</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+3200</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>7436</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+440</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>27957</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+6364</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>15221</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+6383</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>5783</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>15254</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+2980</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>7396</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>560</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>8463</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2260</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:09:48
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -14334,11 +14334,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:00:10</t>
+          <t>Timestamp: 2026-08-17 13:09:48</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>82903</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
@@ -14500,11 +14500,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>26390</v>
+        <v>26460</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+6219</t>
+          <t>+6289</t>
         </is>
       </c>
     </row>
@@ -14695,11 +14695,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>23724</v>
+        <v>23794</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+4980</t>
+          <t>+5050</t>
         </is>
       </c>
     </row>
@@ -14815,11 +14815,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>12743</v>
+        <v>12813</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2560</t>
+          <t>+2630</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:30:22
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -14334,11 +14334,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:09:48</t>
+          <t>Timestamp: 2026-08-17 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>210</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -14605,11 +14605,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>31356</v>
+        <v>31426</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+10160</t>
+          <t>+10230</t>
         </is>
       </c>
     </row>
@@ -14920,11 +14920,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>27957</v>
+        <v>28027</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+6364</t>
+          <t>+6434</t>
         </is>
       </c>
     </row>
@@ -14935,11 +14935,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>15221</v>
+        <v>15291</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+6383</t>
+          <t>+6453</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:40:04
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -14334,11 +14334,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:30:22</t>
+          <t>Timestamp: 2026-08-17 13:40:03</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>420</v>
+        <v>630</v>
       </c>
     </row>
     <row r="3">
@@ -14500,11 +14500,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>26460</v>
+        <v>26530</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+6289</t>
+          <t>+6359</t>
         </is>
       </c>
     </row>
@@ -14605,11 +14605,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>31426</v>
+        <v>31496</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+10230</t>
+          <t>+10300</t>
         </is>
       </c>
     </row>
@@ -14920,11 +14920,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>28027</v>
+        <v>28097</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+6434</t>
+          <t>+6504</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -31,6 +31,7 @@
     <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15147,6 +15148,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-18 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>31434</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2762</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>281</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>8296</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2760</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>14950</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+2303</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1771</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4046</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>29486</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+2956</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2533</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>34671</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3175</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>4110</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Nami</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>25022</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+451</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>24526</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2650</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>26064</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2270</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2984</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>23663</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2140</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2260</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1525</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>14793</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>10279</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1084</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1270</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>9146</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1710</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>31272</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3175</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>17021</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1730</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>5983</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>16074</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8326</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>560</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>9463</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -15178,11 +15178,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-18 13:00:10</t>
+          <t>Timestamp: 2026-08-18 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>31434</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3">
@@ -15449,11 +15449,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>34671</v>
+        <v>34741</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3175</t>
+          <t>+3245</t>
         </is>
       </c>
     </row>
@@ -15524,11 +15524,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>24526</v>
+        <v>24596</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2650</t>
+          <t>+2720</t>
         </is>
       </c>
     </row>
@@ -15539,11 +15539,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>26064</v>
+        <v>26204</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2270</t>
+          <t>+2410</t>
         </is>
       </c>
     </row>
@@ -15569,11 +15569,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>23663</v>
+        <v>23733</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2140</t>
+          <t>+2210</t>
         </is>
       </c>
     </row>
@@ -15689,11 +15689,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>10279</v>
+        <v>10286</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1084</t>
+          <t>+1091</t>
         </is>
       </c>
     </row>
@@ -15749,11 +15749,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>9146</v>
+        <v>9216</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1710</t>
+          <t>+1780</t>
         </is>
       </c>
     </row>
@@ -15764,11 +15764,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>31272</v>
+        <v>31342</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3175</t>
+          <t>+3245</t>
         </is>
       </c>
     </row>
@@ -15809,11 +15809,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>16074</v>
+        <v>16104</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+850</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:34:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -15178,11 +15178,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-18 13:30:22</t>
+          <t>Timestamp: 2026-08-18 13:34:08</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>525</v>
+        <v>595</v>
       </c>
     </row>
     <row r="3">
@@ -15449,11 +15449,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>34741</v>
+        <v>34811</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3245</t>
+          <t>+3315</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:00:12
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -32,6 +32,7 @@
     <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-08-19" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15991,6 +15992,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-19 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25530</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2912</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>6250</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>281</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>8600</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+304</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2760</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>16320</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1370</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1771</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4046</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>31326</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2783</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>38031</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3220</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>4410</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Nami</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>25322</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>26646</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2050</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>28934</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2730</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2984</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>25813</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2080</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2260</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1825</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>16303</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1510</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>10736</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1640</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>10636</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1420</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>34632</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3290</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>18252</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1231</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>6003</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>16904</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8326</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>9963</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:03:42
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16022,11 +16022,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:00:11</t>
+          <t>Timestamp: 2026-08-19 13:03:41</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25530</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -16293,11 +16293,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>38031</v>
+        <v>38101</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3220</t>
+          <t>+3290</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:30:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16022,11 +16022,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:03:41</t>
+          <t>Timestamp: 2026-08-19 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>70</v>
+        <v>620</v>
       </c>
     </row>
     <row r="3">
@@ -16383,11 +16383,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>28934</v>
+        <v>29004</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2730</t>
+          <t>+2800</t>
         </is>
       </c>
     </row>
@@ -16413,11 +16413,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>25813</v>
+        <v>25883</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2080</t>
+          <t>+2150</t>
         </is>
       </c>
     </row>
@@ -16503,11 +16503,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>16303</v>
+        <v>16373</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1510</t>
+          <t>+1580</t>
         </is>
       </c>
     </row>
@@ -16608,11 +16608,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>34632</v>
+        <v>34702</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3290</t>
+          <t>+3360</t>
         </is>
       </c>
     </row>
@@ -16623,11 +16623,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>18252</v>
+        <v>18322</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+1231</t>
+          <t>+1301</t>
         </is>
       </c>
     </row>
@@ -16653,11 +16653,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>16904</v>
+        <v>17104</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:33:57
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16022,11 +16022,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:30:24</t>
+          <t>Timestamp: 2026-08-19 13:33:56</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>620</v>
+        <v>690</v>
       </c>
     </row>
     <row r="3">
@@ -16293,11 +16293,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>38101</v>
+        <v>38171</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3290</t>
+          <t>+3360</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:56:55
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16022,11 +16022,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:33:56</t>
+          <t>Timestamp: 2026-08-19 13:56:54</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>690</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="3">
@@ -16188,11 +16188,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>31326</v>
+        <v>31626</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+1840</t>
+          <t>+2140</t>
         </is>
       </c>
     </row>
@@ -16413,11 +16413,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>25883</v>
+        <v>25953</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2150</t>
+          <t>+2220</t>
         </is>
       </c>
     </row>
@@ -16503,11 +16503,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>16373</v>
+        <v>16443</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1580</t>
+          <t>+1650</t>
         </is>
       </c>
     </row>
@@ -16608,11 +16608,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>34702</v>
+        <v>34772</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3360</t>
+          <t>+3430</t>
         </is>
       </c>
     </row>
@@ -16623,11 +16623,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>18322</v>
+        <v>18392</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+1301</t>
+          <t>+1371</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:04:59
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16866,11 +16866,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:00:10</t>
+          <t>Timestamp: 2026-08-20 13:04:58</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>23569</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -17347,11 +17347,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>18711</v>
+        <v>18781</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2268</t>
+          <t>+2338</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:30:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16866,11 +16866,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:04:58</t>
+          <t>Timestamp: 2026-08-20 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>70</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -17227,11 +17227,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>31198</v>
+        <v>31338</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2194</t>
+          <t>+2334</t>
         </is>
       </c>
     </row>
@@ -17257,11 +17257,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>27893</v>
+        <v>27963</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+1940</t>
+          <t>+2010</t>
         </is>
       </c>
     </row>
@@ -17437,11 +17437,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>12056</v>
+        <v>12126</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1420</t>
+          <t>+1490</t>
         </is>
       </c>
     </row>
@@ -17452,11 +17452,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>37668</v>
+        <v>37738</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2896</t>
+          <t>+2966</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:57:56
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -16866,11 +16866,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:35:12</t>
+          <t>Timestamp: 2026-08-20 13:57:55</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>420</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="3">
@@ -17212,11 +17212,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>29046</v>
+        <v>29246</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -17227,11 +17227,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>31338</v>
+        <v>31378</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2334</t>
+          <t>+2374</t>
         </is>
       </c>
     </row>
@@ -17257,11 +17257,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>27963</v>
+        <v>28033</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2010</t>
+          <t>+2080</t>
         </is>
       </c>
     </row>
@@ -17347,11 +17347,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>18781</v>
+        <v>18851</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2338</t>
+          <t>+2408</t>
         </is>
       </c>
     </row>
@@ -17437,11 +17437,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>12126</v>
+        <v>12196</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1490</t>
+          <t>+1560</t>
         </is>
       </c>
     </row>
@@ -17452,11 +17452,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>37738</v>
+        <v>37808</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2966</t>
+          <t>+3036</t>
         </is>
       </c>
     </row>
@@ -17497,11 +17497,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>17498</v>
+        <v>17698</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+394</t>
+          <t>+594</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -34,6 +34,7 @@
     <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-19" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-08-20" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17679,6 +17680,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-21 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>23459</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2912</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>6550</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>9610</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2760</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>19749</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1771</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4646</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>34755</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+1549</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Third Eye</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2808</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>41151</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1090</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>4410</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>25622</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>31006</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1760</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>34030</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2652</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2984</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>30227</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2194</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2260</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1825</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>20018</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1167</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>11036</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1931</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>200$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>14214</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>40866</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3058</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>20799</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1340</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>6063</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>18368</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8617</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+141</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>11463</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:05:39
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -17710,11 +17710,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:00:10</t>
+          <t>Timestamp: 2026-08-21 13:05:38</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>23459</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3">
@@ -18281,11 +18281,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>14214</v>
+        <v>14234</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+2018</t>
+          <t>+2038</t>
         </is>
       </c>
     </row>
@@ -18296,11 +18296,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>40866</v>
+        <v>40873</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3058</t>
+          <t>+3065</t>
         </is>
       </c>
     </row>
@@ -18311,11 +18311,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>20799</v>
+        <v>20869</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1410</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:30:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -17710,11 +17710,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:05:38</t>
+          <t>Timestamp: 2026-08-21 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>97</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3">
@@ -18056,11 +18056,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>31006</v>
+        <v>31076</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+1760</t>
+          <t>+1830</t>
         </is>
       </c>
     </row>
@@ -18101,11 +18101,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>30227</v>
+        <v>30297</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2194</t>
+          <t>+2264</t>
         </is>
       </c>
     </row>
@@ -18281,11 +18281,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>14234</v>
+        <v>14286</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+2038</t>
+          <t>+2090</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:35:50
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -17710,11 +17710,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:30:24</t>
+          <t>Timestamp: 2026-08-21 13:35:49</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="3">
@@ -18281,11 +18281,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>14286</v>
+        <v>14291</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+2090</t>
+          <t>+2095</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:59:17
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -17710,11 +17710,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:35:49</t>
+          <t>Timestamp: 2026-08-21 13:59:16</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>294</v>
+        <v>765</v>
       </c>
     </row>
     <row r="3">
@@ -18056,11 +18056,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>31076</v>
+        <v>31146</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+1830</t>
+          <t>+1900</t>
         </is>
       </c>
     </row>
@@ -18071,11 +18071,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>34030</v>
+        <v>34221</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2652</t>
+          <t>+2843</t>
         </is>
       </c>
     </row>
@@ -18101,11 +18101,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>30297</v>
+        <v>30367</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2264</t>
+          <t>+2334</t>
         </is>
       </c>
     </row>
@@ -18296,11 +18296,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>40873</v>
+        <v>40943</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3065</t>
+          <t>+3135</t>
         </is>
       </c>
     </row>
@@ -18311,11 +18311,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>20869</v>
+        <v>20939</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+1410</t>
+          <t>+1480</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 05:30:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -18554,11 +18554,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-22 13:00:11</t>
+          <t>Timestamp: 2026-08-22 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>23500</v>
+        <v>11146</v>
       </c>
     </row>
     <row r="3">
@@ -18660,11 +18660,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>2860</v>
+        <v>3000</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>+240</t>
         </is>
       </c>
     </row>
@@ -18915,11 +18915,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>36082</v>
+        <v>36482</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+1861</t>
+          <t>+2261</t>
         </is>
       </c>
     </row>
@@ -18930,11 +18930,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>3154</v>
+        <v>3294</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+170</t>
+          <t>+310</t>
         </is>
       </c>
     </row>
@@ -18975,11 +18975,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>2430</v>
+        <v>2570</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+170</t>
+          <t>+310</t>
         </is>
       </c>
     </row>
@@ -19035,11 +19035,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>22368</v>
+        <v>22508</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2490</t>
         </is>
       </c>
     </row>
@@ -19050,11 +19050,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>2960</v>
+        <v>3100</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+170</t>
+          <t>+310</t>
         </is>
       </c>
     </row>
@@ -19125,11 +19125,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>16831</v>
+        <v>16971</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+2540</t>
+          <t>+2680</t>
         </is>
       </c>
     </row>
@@ -19215,11 +19215,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>300</v>
+        <v>10206</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+10206</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -36,6 +36,7 @@
     <sheet name="2026-08-20" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20210,6 +20211,864 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-23 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>81757</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3512</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>20530</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+13980</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10791</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1181</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>5745</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2745</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>25839</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+4000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2371</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>5537</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>38715</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Third Eye</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3058</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>42071</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5010</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>25622</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>37909</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+4693</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>41722</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+5240</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5899</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2605</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>38219</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+6062</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>5330</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2760</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1635</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Death Service</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>1845</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>25718</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+3210</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>5520</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+2420</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11560</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+524</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2252</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+221</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>721</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>20631</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3660</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>42742</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1169</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>26009</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+3520</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>7313</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>19518</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>631</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>12346</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2140</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ruzzz</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>10159</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>15003</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+2280</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:03:07
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -20241,11 +20241,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:00:11</t>
+          <t>Timestamp: 2026-08-23 13:03:06</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>81757</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:30:26
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -20241,11 +20241,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:03:06</t>
+          <t>Timestamp: 2026-08-23 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3">
@@ -20617,11 +20617,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>41722</v>
+        <v>42002</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+5240</t>
+          <t>+5520</t>
         </is>
       </c>
     </row>
@@ -20647,11 +20647,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>38219</v>
+        <v>38359</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+6062</t>
+          <t>+6202</t>
         </is>
       </c>
     </row>
@@ -20857,11 +20857,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>26009</v>
+        <v>26149</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+3520</t>
+          <t>+3660</t>
         </is>
       </c>
     </row>
@@ -20872,11 +20872,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>7313</v>
+        <v>7453</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1380</t>
         </is>
       </c>
     </row>
@@ -20947,11 +20947,11 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>10159</v>
+        <v>10459</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1460</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:56:18
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -20241,11 +20241,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:33:19</t>
+          <t>Timestamp: 2026-08-23 13:56:17</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1000</v>
+        <v>4490</v>
       </c>
     </row>
     <row r="3">
@@ -20647,11 +20647,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>38359</v>
+        <v>38499</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+6202</t>
+          <t>+6342</t>
         </is>
       </c>
     </row>
@@ -20857,11 +20857,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>26149</v>
+        <v>26289</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+3660</t>
+          <t>+3800</t>
         </is>
       </c>
     </row>
@@ -20872,11 +20872,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>7453</v>
+        <v>7593</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>
@@ -20917,11 +20917,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>12346</v>
+        <v>15416</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2140</t>
+          <t>+5210</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -37,6 +37,7 @@
     <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21069,6 +21070,864 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-24 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>62142</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3612</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>21730</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>11972</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1181</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>28688</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+2849</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2371</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>6137</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>41140</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+2425</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3058</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>44398</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+2327</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5010</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>25622</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>3573</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+3372</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>43249</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+5340</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>47409</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+5407</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2640</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>42167</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+3668</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1360</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>1885</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SS | Lone ™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>La Mujer De Judas</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>27659</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+1941</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1925</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11560</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>4216</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+1964</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>721</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Valenti</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>21431</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>43482</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>28729</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+2440</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>9973</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+2380</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>19518</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+224</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>20199</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+4783</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>11659</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Shimura</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>17586</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+2583</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>568</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>343</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+143</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+340</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:19:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -21100,11 +21100,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:00:09</t>
+          <t>Timestamp: 2026-08-24 13:19:09</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>62142</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3">
@@ -21596,11 +21596,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>27659</v>
+        <v>27829</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+1941</t>
+          <t>+2111</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:30:21
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -21100,11 +21100,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:19:09</t>
+          <t>Timestamp: 2026-08-24 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>170</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3">
@@ -21446,11 +21446,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>43249</v>
+        <v>43389</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+5340</t>
+          <t>+5480</t>
         </is>
       </c>
     </row>
@@ -21596,11 +21596,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>27829</v>
+        <v>27869</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+2111</t>
+          <t>+2151</t>
         </is>
       </c>
     </row>
@@ -21716,11 +21716,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>28729</v>
+        <v>28731</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+2440</t>
+          <t>+2442</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:49:25
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -21100,11 +21100,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:30:21</t>
+          <t>Timestamp: 2026-08-24 13:49:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>352</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="3">
@@ -21476,11 +21476,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>47409</v>
+        <v>47549</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+5407</t>
+          <t>+5547</t>
         </is>
       </c>
     </row>
@@ -21506,11 +21506,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>42167</v>
+        <v>42447</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+3668</t>
+          <t>+3948</t>
         </is>
       </c>
     </row>
@@ -21596,11 +21596,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>27869</v>
+        <v>27939</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+2151</t>
+          <t>+2221</t>
         </is>
       </c>
     </row>
@@ -21716,11 +21716,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>28731</v>
+        <v>28907</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+2442</t>
+          <t>+2618</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -38,6 +38,7 @@
     <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21928,6 +21929,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-25 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25088</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3982</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>22330</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>12744</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+772</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>29588</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Nagasaki</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>191</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2371</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>6437</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>42993</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+1853</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>3299</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+241</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>47157</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2759</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>5301</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+291</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>25622</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>3573</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>45839</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2450</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>49705</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2156</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>44556</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+2109</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1170</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2196</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+311</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>30312</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11860</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>4216</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>791</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+70</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Mercury</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>21861</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+430</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>43992</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>30657</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+1750</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>9993</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>19718</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>21176</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+977</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>11975</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+316</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>19047</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>668</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>560</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:06:22
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -21959,11 +21959,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:00:10</t>
+          <t>Timestamp: 2026-08-25 13:06:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25088</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3">
@@ -22380,11 +22380,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>44556</v>
+        <v>44776</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+2109</t>
+          <t>+2329</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:30:21
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -21959,11 +21959,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:06:21</t>
+          <t>Timestamp: 2026-08-25 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>190</v>
+        <v>960</v>
       </c>
     </row>
     <row r="3">
@@ -22020,11 +22020,11 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>22330</v>
+        <v>22550</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+820</t>
         </is>
       </c>
     </row>
@@ -22320,11 +22320,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>45839</v>
+        <v>45909</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2520</t>
         </is>
       </c>
     </row>
@@ -22350,11 +22350,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>49705</v>
+        <v>49905</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2156</t>
+          <t>+2356</t>
         </is>
       </c>
     </row>
@@ -22455,7 +22455,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>30312</v>
+        <v>30382</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -22545,11 +22545,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>21861</v>
+        <v>21931</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -22635,11 +22635,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>21176</v>
+        <v>21316</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+977</t>
+          <t>+1117</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:58:52
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -21959,11 +21959,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:36:40</t>
+          <t>Timestamp: 2026-08-25 13:58:52</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>960</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="3">
@@ -22320,11 +22320,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>45909</v>
+        <v>45979</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2520</t>
+          <t>+2590</t>
         </is>
       </c>
     </row>
@@ -22380,11 +22380,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>44776</v>
+        <v>44846</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+2329</t>
+          <t>+2399</t>
         </is>
       </c>
     </row>
@@ -22455,7 +22455,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>30382</v>
+        <v>30452</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -22545,11 +22545,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>21931</v>
+        <v>22001</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+570</t>
         </is>
       </c>
     </row>
@@ -22635,11 +22635,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>21316</v>
+        <v>21386</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1117</t>
+          <t>+1187</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -39,6 +39,7 @@
     <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22772,6 +22773,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-26 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22612</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4886</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+904</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>22850</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal Anbu</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>290</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>13114</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>30899</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1311</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Nagasaki</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>273</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+82</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2381</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6437</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>43733</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>3299</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>50017</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+2860</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>5301</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>27243</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1621</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>3573</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>48150</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+2171</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>52058</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+2153</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45126</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1230</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+60</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2196</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>30772</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+320</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>12160</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>4516</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>1391</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Mercury</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>44592</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>30657</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>9993</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>20058</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+340</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>22316</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>12275</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>20537</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1490</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>768</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>543</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>660</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:06:34
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -22803,11 +22803,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:00:10</t>
+          <t>Timestamp: 2026-08-26 13:06:33</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>22612</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -22803,11 +22803,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:06:33</t>
+          <t>Timestamp: 2026-08-26 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -23149,11 +23149,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>27243</v>
+        <v>27313</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+1621</t>
+          <t>+1691</t>
         </is>
       </c>
     </row>
@@ -23179,11 +23179,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>48150</v>
+        <v>48220</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+2171</t>
+          <t>+2241</t>
         </is>
       </c>
     </row>
@@ -23209,11 +23209,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>52058</v>
+        <v>52198</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+2153</t>
+          <t>+2293</t>
         </is>
       </c>
     </row>
@@ -23284,7 +23284,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>1260</v>
+        <v>1330</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -23509,7 +23509,7 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>1260</v>
+        <v>1330</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -40,6 +40,7 @@
     <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23661,6 +23662,879 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-27 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>26316</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>5871</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+985</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23820</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+970</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal Anbu</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1275</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+985</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>13764</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>32659</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1760</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2381</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>6737</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>46083</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>3299</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>50017</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>5301</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>29880</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+2567</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>STARBOY MR. K</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>3573</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>50410</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2190</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2802</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>45126</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1230</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>3870</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+2540</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2346</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>30822</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>12451</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+291</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>4516</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>1391</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Mercury</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>47281</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+2689</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>30657</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>10013</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>20388</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+330</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>3467</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2137</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>23066</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>12575</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>21247</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>938</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>643</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 05:30:21
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -23692,11 +23692,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-27 13:00:09</t>
+          <t>Timestamp: 2026-08-27 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>26316</v>
+        <v>710</v>
       </c>
     </row>
     <row r="3">
@@ -23753,11 +23753,11 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>23820</v>
+        <v>24120</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+1270</t>
         </is>
       </c>
     </row>
@@ -24053,11 +24053,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>50410</v>
+        <v>50480</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+2190</t>
+          <t>+2260</t>
         </is>
       </c>
     </row>
@@ -24083,11 +24083,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>55000</v>
+        <v>55070</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2802</t>
+          <t>+2872</t>
         </is>
       </c>
     </row>
@@ -24308,11 +24308,11 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>47281</v>
+        <v>47351</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+2689</t>
+          <t>+2759</t>
         </is>
       </c>
     </row>
@@ -24353,11 +24353,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>20388</v>
+        <v>20588</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+530</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -41,6 +41,7 @@
     <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24535,6 +24536,864 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-28 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>24374</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6382</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+511</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>24360</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+240</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal Anbu</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+481</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>13764</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>34551</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1892</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2381</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>6737</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>46444</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+361</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>3299</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>51079</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1062</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>5401</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>29880</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>52521</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2041</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>57462</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+2392</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>45236</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+110</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1230</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6841</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+2971</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2346</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>31182</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>12751</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>4716</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>1391</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>50596</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+3245</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>30657</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>10103</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+90</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>21799</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1211</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>5901</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2434</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>24118</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1052</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>13025</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>22868</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+1621</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1108</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>813</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -24566,11 +24566,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-28 13:00:10</t>
+          <t>Timestamp: 2026-08-28 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>24374</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3">
@@ -24912,11 +24912,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>52521</v>
+        <v>52591</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2041</t>
+          <t>+2111</t>
         </is>
       </c>
     </row>
@@ -25032,11 +25032,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>6841</v>
+        <v>6911</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+2971</t>
+          <t>+3041</t>
         </is>
       </c>
     </row>
@@ -25167,11 +25167,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>50596</v>
+        <v>50599</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+3245</t>
+          <t>+3248</t>
         </is>
       </c>
     </row>
@@ -25242,11 +25242,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>5901</v>
+        <v>5971</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2434</t>
+          <t>+2504</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:33:32
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -24566,11 +24566,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-28 13:30:22</t>
+          <t>Timestamp: 2026-08-28 13:33:31</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>213</v>
+        <v>305</v>
       </c>
     </row>
     <row r="3">
@@ -25167,11 +25167,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>50599</v>
+        <v>50691</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+3248</t>
+          <t>+3340</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -42,6 +42,7 @@
     <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25394,6 +25395,864 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-29 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25410</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Naligord</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kyousuke </t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>6532</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>24660</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS Thomas Shelby</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal Anbu</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1906</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>14424</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>34851</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2381</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>7037</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>46444</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1180</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MUSIBAT/0.5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>168</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>5150</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>3299</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>51079</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>5401</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Asuna Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>31810</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+1930</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>54644</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2053</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>59974</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+2512</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>46206</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+970</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>1240</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>9193</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+2282</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2675</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+40</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2356</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>31182</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>12751</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>5278</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+562</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>1391</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>53866</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+3175</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>32000</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+1343</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>10143</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+40</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>22642</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+843</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>855</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8291</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2320</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>xZenny V</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>25962</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+1844</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>13695</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>benji</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>24539</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+1671</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1083</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+270</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:30:22
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -25425,11 +25425,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:00:09</t>
+          <t>Timestamp: 2026-08-29 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25410</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="3">
@@ -25531,11 +25531,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>14424</v>
+        <v>14564</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+800</t>
         </is>
       </c>
     </row>
@@ -25771,11 +25771,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>54644</v>
+        <v>54784</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+2053</t>
+          <t>+2193</t>
         </is>
       </c>
     </row>
@@ -25801,11 +25801,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>59974</v>
+        <v>60174</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+2512</t>
+          <t>+2712</t>
         </is>
       </c>
     </row>
@@ -25846,11 +25846,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>46206</v>
+        <v>46346</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+1110</t>
         </is>
       </c>
     </row>
@@ -25876,11 +25876,11 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>6690</v>
+        <v>6771</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+81</t>
         </is>
       </c>
     </row>
@@ -26026,11 +26026,11 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>53866</v>
+        <v>54006</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>+3175</t>
+          <t>+3315</t>
         </is>
       </c>
     </row>
@@ -26116,11 +26116,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>25962</v>
+        <v>27262</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+1844</t>
+          <t>+3144</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-30 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -43,6 +43,7 @@
     <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26253,6 +26254,789 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-30 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>27605</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>44487</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+19827</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23515</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>28678</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+14114</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10376</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+2831</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>53873</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+19022</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>24652</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+22271</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>28399</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+21362</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>63100</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+16656</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>24538</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+23358</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>17645</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+17145</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>25638</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+20488</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>17948</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>6198</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+4988</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>73517</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+22438</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>5401</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>35471</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+3661</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>77075</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+22291</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>9448</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+9448</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>69213</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+9039</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>19058</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+18908</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>10579</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+2040</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>53231</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+6885</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>9134</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2363</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>25329</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+16136</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>19777</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+17102</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>20764</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+18408</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>45476</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+14294</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>10450</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+3005</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>31848</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+19097</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>27167</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+21889</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21942</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+20551</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7816</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>83702</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+29696</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>36813</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+4813</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>19369</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+9226</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>37882</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+15240</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>13520</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+5229</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>50776</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>18235</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+18035</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36353</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+22658</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>18663</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+17703</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>41659</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+17120</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>18947</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+17639</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>16337</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+15254</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>17085</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+15925</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-31 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27037,6 +27038,789 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-31 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>27605</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>44487</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23515</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>28678</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10376</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>53873</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>24652</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>28399</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>63100</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>24538</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>17645</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>25638</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>17948</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>6198</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>73517</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>5401</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>35471</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>77075</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>9448</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>69213</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>19058</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>10579</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>53231</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>9134</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>25329</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>19777</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>20764</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>45476</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>10450</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>31848</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>27167</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21942</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7816</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>83702</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>36813</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>19369</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>37882</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>13520</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>50776</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>18235</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36353</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>18663</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>41659</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>18947</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>16337</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>17085</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-01 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -45,6 +45,7 @@
     <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27821,6 +27822,789 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-01 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>27605</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>44487</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23515</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>28678</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>10376</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>53873</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>24652</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>28399</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>63100</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>24538</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>17645</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>25638</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>17948</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>6198</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>73517</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>5401</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>35471</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>77075</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>9448</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>69213</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>19058</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>10579</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>53231</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>9134</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>25329</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>19777</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>20764</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>45476</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>10450</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>31848</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>27167</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21942</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7816</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>22151</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>83702</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>36813</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>19369</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>37882</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>13520</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>50776</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>18235</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36353</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>18663</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>41659</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>18947</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>16337</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>17085</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -46,6 +46,7 @@
     <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29463,6 +29464,789 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-02 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>194</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>146</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>295</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 05:30:32
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -29494,11 +29494,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-02 13:00:10</t>
+          <t>Timestamp: 2026-09-02 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>701</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="3">
@@ -29780,7 +29780,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0</v>
+        <v>404</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -29795,7 +29795,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>194</v>
+        <v>224</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
@@ -29900,7 +29900,7 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>0</v>
+        <v>388</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
@@ -30110,7 +30110,7 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>0</v>
+        <v>242</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
@@ -30185,7 +30185,7 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>0</v>
+        <v>494</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 05:00:11
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -47,6 +47,7 @@
     <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30247,6 +30248,804 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-03 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25390</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>355</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+355</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS | Ali Fka</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4388</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+4388</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>954</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+954</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1940</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2566</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+2162</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2168</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1944</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>1386</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>294</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+294</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2331</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1943</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>513</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+513</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SETYA:) </t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>182</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+182</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+2635</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS HaN</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>295</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2047</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+1805</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>417</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+417</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 05:30:27
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -30278,11 +30278,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-03 13:00:10</t>
+          <t>Timestamp: 2026-09-03 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25390</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3">
@@ -30429,11 +30429,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>4388</v>
+        <v>4438</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+4388</t>
+          <t>+4438</t>
         </is>
       </c>
     </row>
@@ -30504,11 +30504,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>954</v>
+        <v>1004</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+954</t>
+          <t>+1004</t>
         </is>
       </c>
     </row>
@@ -30579,11 +30579,11 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>2566</v>
+        <v>2616</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>+2162</t>
+          <t>+2212</t>
         </is>
       </c>
     </row>
@@ -30594,11 +30594,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>2168</v>
+        <v>2218</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+1944</t>
+          <t>+1994</t>
         </is>
       </c>
     </row>
@@ -30699,11 +30699,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>2331</v>
+        <v>2381</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1943</t>
+          <t>+1993</t>
         </is>
       </c>
     </row>
@@ -30849,11 +30849,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>2635</v>
+        <v>2685</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+2635</t>
+          <t>+2685</t>
         </is>
       </c>
     </row>
@@ -30909,11 +30909,11 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>2047</v>
+        <v>2097</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>+1805</t>
+          <t>+1855</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 05:30:26
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -31077,11 +31077,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-04 13:00:12</t>
+          <t>Timestamp: 2026-09-04 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25756</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -31648,11 +31648,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>806</v>
+        <v>856</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+806</t>
+          <t>+856</t>
         </is>
       </c>
     </row>
@@ -31663,11 +31663,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>4634</v>
+        <v>4684</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+1949</t>
+          <t>+1999</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -49,6 +49,7 @@
     <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31845,6 +31846,804 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-05 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>29472</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>366</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>682</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+82</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2838</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1460</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1255</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>18077</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+7136</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>225</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3232</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1181</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>8876</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2189</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>5549</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1482</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>5144</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+1230</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>2993</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1407</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+1401</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>5315</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1512</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>949</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>360</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+40</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 196$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>530</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+955</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>6728</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+2044</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>882</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>5087</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+1635</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>921</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+816</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>2936</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1027</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 05:30:20
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -31876,11 +31876,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-05 13:00:08</t>
+          <t>Timestamp: 2026-09-05 13:30:19</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>29472</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3">
@@ -32237,11 +32237,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>2993</v>
+        <v>3193</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+1407</t>
+          <t>+1607</t>
         </is>
       </c>
     </row>
@@ -32282,11 +32282,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+1401</t>
+          <t>+1501</t>
         </is>
       </c>
     </row>
@@ -32432,11 +32432,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>1137</v>
+        <v>1180</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+955</t>
+          <t>+998</t>
         </is>
       </c>
     </row>
@@ -32462,11 +32462,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>6728</v>
+        <v>6828</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+2044</t>
+          <t>+2144</t>
         </is>
       </c>
     </row>
@@ -32552,11 +32552,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+816</t>
+          <t>+820</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -50,6 +50,7 @@
     <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32644,6 +32645,819 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-06 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>55517</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>576</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1063</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+643</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>681</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+381</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SS MAK LAMPIR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>682</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2855</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+2855</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>3829</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+991</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1255</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>19699</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1622</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>385</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+160</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2810</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+2810</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3232</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>10598</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1722</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>7281</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1732</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>8849</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+3705</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>4553</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1360</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>2831</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2831</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>7125</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+5325</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>3098</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+3098</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>8435</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+3120</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>430</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>1709</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2098</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2098</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1970</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 196$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>530</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>1829</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+649</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>3404</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1748</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>11097</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+4269</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>882</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>7897</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+2810</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>5449</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+3049</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>3025</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>5098</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+2162</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+110</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 05:30:21
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -32675,11 +32675,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-06 13:00:09</t>
+          <t>Timestamp: 2026-09-06 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>55517</v>
+        <v>3054</v>
       </c>
     </row>
     <row r="3">
@@ -32706,11 +32706,11 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>576</v>
+        <v>876</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>+210</t>
+          <t>+510</t>
         </is>
       </c>
     </row>
@@ -32736,11 +32736,11 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>681</v>
+        <v>981</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>+381</t>
+          <t>+681</t>
         </is>
       </c>
     </row>
@@ -32901,11 +32901,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>2810</v>
+        <v>2860</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+2810</t>
+          <t>+2860</t>
         </is>
       </c>
     </row>
@@ -33006,11 +33006,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>8849</v>
+        <v>8949</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+3705</t>
+          <t>+3805</t>
         </is>
       </c>
     </row>
@@ -33066,11 +33066,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2831</v>
+        <v>2931</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2831</t>
+          <t>+2931</t>
         </is>
       </c>
     </row>
@@ -33081,11 +33081,11 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>7125</v>
+        <v>7175</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>+5325</t>
+          <t>+5375</t>
         </is>
       </c>
     </row>
@@ -33096,11 +33096,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>3098</v>
+        <v>3198</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+3098</t>
+          <t>+3198</t>
         </is>
       </c>
     </row>
@@ -33156,11 +33156,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>1709</v>
+        <v>1833</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+884</t>
         </is>
       </c>
     </row>
@@ -33171,11 +33171,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>2098</v>
+        <v>2198</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+2098</t>
+          <t>+2198</t>
         </is>
       </c>
     </row>
@@ -33231,11 +33231,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>1829</v>
+        <v>1979</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+649</t>
+          <t>+799</t>
         </is>
       </c>
     </row>
@@ -33246,11 +33246,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>3404</v>
+        <v>3454</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1748</t>
+          <t>+1798</t>
         </is>
       </c>
     </row>
@@ -33261,11 +33261,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>11097</v>
+        <v>11147</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+4269</t>
+          <t>+4319</t>
         </is>
       </c>
     </row>
@@ -33336,11 +33336,11 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>5449</v>
+        <v>7029</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>+3049</t>
+          <t>+4629</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -51,6 +51,7 @@
     <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33458,6 +33459,819 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-07 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>48264</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1176</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1063</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3305</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5171</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1342</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1555</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>20838</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1139</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>505</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+120</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>3260</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4082</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>11684</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1086</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>9191</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+1910</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>11205</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+2256</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>4953</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3181</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>9785</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2610</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>3412</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+214</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>11115</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+2680</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>430</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>4850</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+3017</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>5926</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+3596</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>3015</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 196$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>953</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+423</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>5604</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+3625</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>6074</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+2620</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>14602</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+3455</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1142</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+260</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>9819</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1922</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>8569</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+1540</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>5305</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2280</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>6598</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>210</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 05:30:21
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -33468,7 +33468,7 @@
   <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -33489,11 +33489,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-07 13:00:08</t>
+          <t>Timestamp: 2026-09-07 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>48264</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3">
@@ -33651,7 +33651,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>SS Aiko Turbo</t>
+          <t>SS Aiko Turbo Saetta</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -33715,11 +33715,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>4082</v>
+        <v>4107</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -33880,11 +33880,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>9785</v>
+        <v>9810</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2610</t>
+          <t>+2635</t>
         </is>
       </c>
     </row>
@@ -33955,11 +33955,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>4850</v>
+        <v>4867</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+3017</t>
+          <t>+3034</t>
         </is>
       </c>
     </row>
@@ -34000,7 +34000,7 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>3015</v>
+        <v>3065</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
@@ -34045,11 +34045,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>5604</v>
+        <v>5625</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+3625</t>
+          <t>+3646</t>
         </is>
       </c>
     </row>
@@ -34060,11 +34060,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>6074</v>
+        <v>6099</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+2620</t>
+          <t>+2645</t>
         </is>
       </c>
     </row>
@@ -34075,11 +34075,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>14602</v>
+        <v>14627</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+3455</t>
+          <t>+3480</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 05:03:24
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -52,6 +52,7 @@
     <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34272,6 +34273,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-08 13:03:22</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1307</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+131</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1248</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+185</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Dajjal</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1413</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+132</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3305</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5746</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1555</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>22005</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1167</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>505</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>3260</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4705</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+598</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>12214</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+530</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>265</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+265</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>9191</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>12410</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1205</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>5494</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+541</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3181</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>11625</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1815</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>3412</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>12035</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>440</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6824</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1957</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6161</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+235</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>4302</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1237</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Setya:) 196$</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+216</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>7223</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+1598</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>7885</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1786</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>16105</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+1478</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1387</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+245</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>10629</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>8569</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>5680</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>6828</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+230</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>229</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+19</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1126</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 05:33:37
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -34303,11 +34303,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-08 13:03:22</t>
+          <t>Timestamp: 2026-09-08 13:33:35</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
@@ -34694,11 +34694,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>11625</v>
+        <v>11655</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+1815</t>
+          <t>+1845</t>
         </is>
       </c>
     </row>
@@ -34769,11 +34769,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>6824</v>
+        <v>6864</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+1957</t>
+          <t>+1997</t>
         </is>
       </c>
     </row>
@@ -34859,11 +34859,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>7223</v>
+        <v>7253</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+1598</t>
+          <t>+1628</t>
         </is>
       </c>
     </row>
@@ -34874,11 +34874,11 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>7885</v>
+        <v>7915</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+1786</t>
+          <t>+1816</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-09 05:00:14
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -53,6 +53,7 @@
     <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35101,6 +35102,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-09 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>24692</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Satanouske</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1672</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+365</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1248</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Kyoustanic</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1793</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3305</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7355</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1609</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1855</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>23691</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1686</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>580</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>650</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>3260</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>5431</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+726</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>12657</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+443</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>265</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>9191</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>13953</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+1543</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6249</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+755</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>3181</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>13635</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>3412</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>12785</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>8027</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1163</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>6161</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>5988</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1686</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>SETYA:)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>9182</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+1929</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>9780</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+1865</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>18511</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+2406</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1627</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+240</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>11158</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+529</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>8569</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>5980</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>7878</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>279</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1322</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -54,6 +54,7 @@
     <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35915,6 +35916,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-10 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>21765</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1548</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3305</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>8796</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+1441</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1855</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>25505</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1764</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>580</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>650</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>3260</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>6195</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+714</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>13262</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>2640</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+1715</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>772</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+507</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>9191</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>290</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>15758</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1805</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>BOBOYBLAZE</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>6849</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3181</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>15872</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+2137</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>3412</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>12885</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8127</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>6811</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>7811</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1823</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SETYA:)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>11396</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+2114</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>9780</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>19011</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1887</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+260</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>11863</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+705</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>8869</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>5980</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>9073</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1195</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>3868</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1420</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 05:30:23
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -35946,11 +35946,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-10 13:00:09</t>
+          <t>Timestamp: 2026-09-10 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>21765</v>
+        <v>610</v>
       </c>
     </row>
     <row r="3">
@@ -36052,11 +36052,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>25505</v>
+        <v>25605</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+1764</t>
+          <t>+1864</t>
         </is>
       </c>
     </row>
@@ -36142,11 +36142,11 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>6195</v>
+        <v>6245</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>+714</t>
+          <t>+764</t>
         </is>
       </c>
     </row>
@@ -36202,11 +36202,11 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>2640</v>
+        <v>2690</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>+1715</t>
+          <t>+1765</t>
         </is>
       </c>
     </row>
@@ -36337,11 +36337,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>15872</v>
+        <v>15922</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2137</t>
+          <t>+2187</t>
         </is>
       </c>
     </row>
@@ -36457,11 +36457,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>7811</v>
+        <v>7871</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+1823</t>
+          <t>+1883</t>
         </is>
       </c>
     </row>
@@ -36667,11 +36667,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>9073</v>
+        <v>9373</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+1195</t>
+          <t>+1495</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 05:30:38
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -36775,11 +36775,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-11 13:00:11</t>
+          <t>Timestamp: 2026-09-11 13:30:37</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>24749</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
@@ -36881,11 +36881,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>27469</v>
+        <v>27510</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+1864</t>
+          <t>+1905</t>
         </is>
       </c>
     </row>
@@ -37121,11 +37121,11 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>8049</v>
+        <v>8052</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1203</t>
         </is>
       </c>
     </row>
@@ -37166,11 +37166,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>18200</v>
+        <v>18224</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+2278</t>
+          <t>+2302</t>
         </is>
       </c>
     </row>
@@ -37361,11 +37361,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>20384</v>
+        <v>20434</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+1373</t>
+          <t>+1423</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 05:00:09
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -56,6 +56,7 @@
     <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38431,6 +38432,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-12 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22013</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1848</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3305</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>11689</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+1429</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2455</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>29052</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1542</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>580</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>941</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+291</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>3360</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>7236</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>16645</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1679</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>5487</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+1451</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1864</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+519</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>9191</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>1363</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+132</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>19377</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+1650</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>2041</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>9355</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+1303</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3311</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+130</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>19247</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1023</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>3412</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>13968</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8127</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2448</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>7722</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>11502</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+1741</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SETYA:)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>11406</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>9790</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>22622</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+2188</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1967</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>13432</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1128</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>10065</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>7181</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+237</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>10473</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>629</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>700</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>6300</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1441</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 05:30:51
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -38462,11 +38462,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-12 13:30:23</t>
+          <t>Timestamp: 2026-09-12 13:30:50</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2900</v>
+        <v>2901</v>
       </c>
     </row>
     <row r="3">
@@ -39018,11 +39018,11 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>11706</v>
+        <v>11707</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>+310</t>
+          <t>+311</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 05:00:10
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -57,6 +57,7 @@
     <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39260,6 +39261,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shinigami Secret (3761) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-13 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>54127</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SS Finotxi</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1848</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Tu Verdadero Marido</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4685</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+1180</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>§azacel§</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>13599</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+1910</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>soifon</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mr.1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>3055</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Lokajaya R°</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>31682</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2030</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SS PHARAONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>580</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SS Aiko Turbo Saetta</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>king izzy |Shimura|</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1131</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+190</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ilham</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gata Only</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>4477</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+1117</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Parakang</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>9675</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+2439</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>•R¥U•</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Sakera S1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>18332</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1087</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Anbu Terumi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>8378</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+2691</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Whymeee</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>2854</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evana Van Stenberg </t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>9191</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lagoony</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>1963</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>•Yµmíko•</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>22927</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+3550</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ali Fka Reseller NR</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>4597</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+2456</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ÐictatøR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>11755</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DONQOUIXTE </t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Shinigami Lover</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>4416</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1105</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SS IMORTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>21217</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+1970</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>El Temach</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>4612</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Syu Revenoir</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>14630</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+662</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>LorD</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SS Lone Death</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>990</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SS Master SS </t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8127</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Light Yagami</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>3711</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1063</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Alvaro_DR</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>10294</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2572</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>[N]epotizMe*</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>15313</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+3811</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>RyExHinzxc</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SETYA:)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Cosmo Raion</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>14257</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+2550</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Soul Anbu</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>9940</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dracht</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>26858</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+4136</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SS | german.s97</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gómez </t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2367</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>bjorn</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Zannpist Revenoir</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>14974</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+1542</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>-Supreme Zeno-</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>11645</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+1580</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SS Rain</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SS Ruzzz.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>8081</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>geri</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Itachi Uchiha</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>10803</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+330</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Haruka Sakura</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>829</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Inosuke Hashibira</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Kurosaki Ichigo</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>550</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>elmacho</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>9775</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+3475</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 05:30:26
</commit_message>
<xml_diff>
--- a/clan_3761.xlsx
+++ b/clan_3761.xlsx
@@ -39291,11 +39291,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-13 13:00:08</t>
+          <t>Timestamp: 2026-09-13 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54127</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3">
@@ -39487,11 +39487,11 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>9675</v>
+        <v>9725</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>+2439</t>
+          <t>+2489</t>
         </is>
       </c>
     </row>
@@ -39607,11 +39607,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>22927</v>
+        <v>22977</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+3550</t>
+          <t>+3600</t>
         </is>
       </c>
     </row>
@@ -39802,11 +39802,11 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>15313</v>
+        <v>15363</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>+3811</t>
+          <t>+3861</t>
         </is>
       </c>
     </row>
@@ -39877,11 +39877,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>26858</v>
+        <v>26908</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+4136</t>
+          <t>+4186</t>
         </is>
       </c>
     </row>

</xml_diff>